<commit_message>
Update public event data
</commit_message>
<xml_diff>
--- a/data/events.xlsx
+++ b/data/events.xlsx
@@ -180,12 +180,12 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:36Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -272,12 +272,12 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:37Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -364,12 +364,12 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:54Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -456,12 +456,12 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:35Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -503,12 +503,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-05-26T20:00:00Z</t>
+          <t>2026-05-26T20:00:00</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-06-02T20:00:00Z</t>
+          <t>2026-06-02T20:00:00</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -548,12 +548,12 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:36Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -640,12 +640,12 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:37Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -732,12 +732,12 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:38Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -779,12 +779,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-05-29T01:00:00Z</t>
+          <t>2026-05-29T01:00:00</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-06-01T11:00:00Z</t>
+          <t>2026-06-01T11:00:00</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -824,12 +824,12 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:35Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -871,7 +871,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-05-31T01:00:00Z</t>
+          <t>2026-05-31T01:00:00</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -916,12 +916,12 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:34Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
@@ -1008,12 +1008,12 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:55Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
@@ -1100,12 +1100,12 @@
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:55Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
@@ -1192,12 +1192,12 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:55Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
@@ -1284,12 +1284,12 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:55Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
@@ -1376,12 +1376,12 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:36Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
@@ -1468,12 +1468,12 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:55Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
@@ -1515,12 +1515,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-06-02T20:00:00Z</t>
+          <t>2026-06-02T20:00:00</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026-06-09T20:00:00Z</t>
+          <t>2026-06-09T20:00:00</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1560,12 +1560,12 @@
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:39Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -1652,12 +1652,12 @@
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:56Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
@@ -1744,12 +1744,12 @@
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:56Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
@@ -1836,12 +1836,12 @@
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:56Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
@@ -1928,12 +1928,12 @@
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:38Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
@@ -2020,12 +2020,12 @@
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:57Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
@@ -2112,12 +2112,12 @@
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:57Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
@@ -2159,12 +2159,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-06-09T20:00:00Z</t>
+          <t>2026-06-09T20:00:00</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>2026-06-16T20:00:00Z</t>
+          <t>2026-06-16T20:00:00</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2204,12 +2204,12 @@
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:42Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
@@ -2296,12 +2296,12 @@
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:57Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
@@ -2388,12 +2388,12 @@
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:57Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
@@ -2480,12 +2480,12 @@
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:57Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
@@ -2572,12 +2572,12 @@
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:41Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
@@ -2664,12 +2664,12 @@
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:58Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
@@ -2711,12 +2711,12 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>2026-06-16T20:00:00Z</t>
+          <t>2026-06-16T20:00:00</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>2026-06-23T20:00:00Z</t>
+          <t>2026-06-23T20:00:00</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2756,12 +2756,12 @@
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:44Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
@@ -2848,12 +2848,12 @@
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:58Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
@@ -2940,12 +2940,12 @@
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:58Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
@@ -3032,12 +3032,12 @@
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:58Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
@@ -3124,12 +3124,12 @@
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:59Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
@@ -3216,12 +3216,12 @@
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:59Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
@@ -3308,12 +3308,12 @@
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:59Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
@@ -3355,12 +3355,12 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>2026-06-23T20:00:00Z</t>
+          <t>2026-06-23T20:00:00</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>2026-06-30T20:00:00Z</t>
+          <t>2026-06-30T20:00:00</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -3400,12 +3400,12 @@
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:47Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
@@ -3492,12 +3492,12 @@
       </c>
       <c r="P38" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:59Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
@@ -3584,12 +3584,12 @@
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:00Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
@@ -3676,12 +3676,12 @@
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:00Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R40" t="inlineStr">
@@ -3768,12 +3768,12 @@
       </c>
       <c r="P41" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:00Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
@@ -3860,12 +3860,12 @@
       </c>
       <c r="P42" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:00Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R42" t="inlineStr">
@@ -3952,12 +3952,12 @@
       </c>
       <c r="P43" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:01Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R43" t="inlineStr">
@@ -3999,12 +3999,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>2026-06-30T20:00:00Z</t>
+          <t>2026-06-30T20:00:00</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>2026-07-07T20:00:00Z</t>
+          <t>2026-07-07T20:00:00</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -4044,12 +4044,12 @@
       </c>
       <c r="P44" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:49Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R44" t="inlineStr">
@@ -4136,12 +4136,12 @@
       </c>
       <c r="P45" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:01Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R45" t="inlineStr">
@@ -4183,12 +4183,12 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>2026-07-07T20:00:00Z</t>
+          <t>2026-07-07T20:00:00</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>2026-07-14T20:00:00Z</t>
+          <t>2026-07-14T20:00:00</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -4228,12 +4228,12 @@
       </c>
       <c r="P46" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:49Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R46" t="inlineStr">
@@ -4320,12 +4320,12 @@
       </c>
       <c r="P47" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:01Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R47" t="inlineStr">
@@ -4367,12 +4367,12 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>2026-07-14T20:00:00Z</t>
+          <t>2026-07-14T20:00:00</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>2026-07-21T20:00:00Z</t>
+          <t>2026-07-21T20:00:00</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -4412,12 +4412,12 @@
       </c>
       <c r="P48" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:50Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
@@ -4504,12 +4504,12 @@
       </c>
       <c r="P49" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:02Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R49" t="inlineStr">
@@ -4551,12 +4551,12 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>2026-07-21T20:00:00Z</t>
+          <t>2026-07-21T20:00:00</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>2026-07-28T20:00:00Z</t>
+          <t>2026-07-28T20:00:00</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -4596,12 +4596,12 @@
       </c>
       <c r="P50" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:50Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
@@ -4643,12 +4643,12 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>2026-07-28T20:00:00Z</t>
+          <t>2026-07-28T20:00:00</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>2026-08-04T20:00:00Z</t>
+          <t>2026-08-04T20:00:00</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -4688,12 +4688,12 @@
       </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:51Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
@@ -4735,12 +4735,12 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>2026-08-04T20:00:00Z</t>
+          <t>2026-08-04T20:00:00</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>2026-08-11T20:00:00Z</t>
+          <t>2026-08-11T20:00:00</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -4780,12 +4780,12 @@
       </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:51Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R52" t="inlineStr">
@@ -4872,12 +4872,12 @@
       </c>
       <c r="P53" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:02Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
@@ -4919,12 +4919,12 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>2026-08-11T20:00:00Z</t>
+          <t>2026-08-11T20:00:00</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>2026-08-18T20:00:00Z</t>
+          <t>2026-08-18T20:00:00</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -4964,12 +4964,12 @@
       </c>
       <c r="P54" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:52Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
@@ -5056,12 +5056,12 @@
       </c>
       <c r="P55" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:02Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
@@ -5103,12 +5103,12 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>2026-08-18T20:00:00Z</t>
+          <t>2026-08-18T20:00:00</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>2026-08-25T20:00:00Z</t>
+          <t>2026-08-25T20:00:00</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -5148,12 +5148,12 @@
       </c>
       <c r="P56" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:53Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R56" t="inlineStr">
@@ -5240,12 +5240,12 @@
       </c>
       <c r="P57" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R57" t="inlineStr">
@@ -5287,12 +5287,12 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>2026-08-25T20:00:00Z</t>
+          <t>2026-08-25T20:00:00</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>2026-09-01T20:00:00Z</t>
+          <t>2026-09-01T20:00:00</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -5332,12 +5332,12 @@
       </c>
       <c r="P58" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:53Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R58" t="inlineStr">
@@ -5379,12 +5379,12 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>2026-09-01T20:00:00Z</t>
+          <t>2026-09-01T20:00:00</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>2026-09-08T20:00:00Z</t>
+          <t>2026-09-08T20:00:00</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -5424,12 +5424,12 @@
       </c>
       <c r="P59" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:54Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R59" t="inlineStr">
@@ -5516,12 +5516,12 @@
       </c>
       <c r="P60" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q60" t="inlineStr">
         <is>
-          <t>2026-05-31T06:38:54Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R60" t="inlineStr">
@@ -5608,12 +5608,12 @@
       </c>
       <c r="P61" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="Q61" t="inlineStr">
         <is>
-          <t>2026-05-31T06:39:03Z</t>
+          <t>2026-05-31T06:40:26Z</t>
         </is>
       </c>
       <c r="R61" t="inlineStr">

</xml_diff>